<commit_message>
Corrección de gráficos del Dashboard: OEE con 8 barras individuales y escala 60-100%
- Gráfico OEE: cada equipo ahora tiene su propia barra coloreada según nivel (verde/amarillo/rojo)
  usando DataPoint individual, escala X ajustada a 60-100% para mostrar la variación real
- Pareto: dimensiones aumentadas para mejor legibilidad
- Datos auxiliares OEE reubicados a columnas 6-7 para evitar colisión con datos del Pareto
</commit_message>
<xml_diff>
--- a/proyectos/excel/gestion-paros-productividad-manufactura/output/Panel_Paros_OEE_Portfolio.xlsx
+++ b/proyectos/excel/gestion-paros-productividad-manufactura/output/Panel_Paros_OEE_Portfolio.xlsx
@@ -645,25 +645,110 @@
           <order val="0"/>
           <tx>
             <strRef>
-              <f>'Dashboard'!B55</f>
+              <f>'Dashboard'!G55</f>
             </strRef>
           </tx>
           <spPr>
-            <a:solidFill>
-              <a:srgbClr val="70AD47"/>
-            </a:solidFill>
             <a:ln>
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
+          <dPt>
+            <idx val="0"/>
+            <spPr>
+              <a:solidFill>
+                <a:srgbClr val="70AD47"/>
+              </a:solidFill>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </dPt>
+          <dPt>
+            <idx val="1"/>
+            <spPr>
+              <a:solidFill>
+                <a:srgbClr val="FFD966"/>
+              </a:solidFill>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </dPt>
+          <dPt>
+            <idx val="2"/>
+            <spPr>
+              <a:solidFill>
+                <a:srgbClr val="FFD966"/>
+              </a:solidFill>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </dPt>
+          <dPt>
+            <idx val="3"/>
+            <spPr>
+              <a:solidFill>
+                <a:srgbClr val="70AD47"/>
+              </a:solidFill>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </dPt>
+          <dPt>
+            <idx val="4"/>
+            <spPr>
+              <a:solidFill>
+                <a:srgbClr val="FFD966"/>
+              </a:solidFill>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </dPt>
+          <dPt>
+            <idx val="5"/>
+            <spPr>
+              <a:solidFill>
+                <a:srgbClr val="FFD966"/>
+              </a:solidFill>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </dPt>
+          <dPt>
+            <idx val="6"/>
+            <spPr>
+              <a:solidFill>
+                <a:srgbClr val="FFD966"/>
+              </a:solidFill>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </dPt>
+          <dPt>
+            <idx val="7"/>
+            <spPr>
+              <a:solidFill>
+                <a:srgbClr val="70AD47"/>
+              </a:solidFill>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </dPt>
           <cat>
             <numRef>
-              <f>'Dashboard'!$A$56:$A$63</f>
+              <f>'Dashboard'!$F$56:$F$63</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Dashboard'!$B$56:$B$63</f>
+              <f>'Dashboard'!$G$56:$G$63</f>
             </numRef>
           </val>
         </ser>
@@ -676,7 +761,7 @@
         <scaling>
           <orientation val="minMax"/>
           <max val="1"/>
-          <min val="0"/>
+          <min val="0.6"/>
         </scaling>
         <axPos val="l"/>
         <title>
@@ -745,7 +830,7 @@
       <row>6</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="6480000" cy="4320000"/>
+    <ext cx="7200000" cy="5040000"/>
     <graphicFrame>
       <nvGraphicFramePr>
         <cNvPr id="1" name="Chart 1"/>
@@ -767,7 +852,7 @@
       <row>6</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="6480000" cy="4320000"/>
+    <ext cx="7920000" cy="5040000"/>
     <graphicFrame>
       <nvGraphicFramePr>
         <cNvPr id="2" name="Chart 2"/>
@@ -1097,25 +1182,27 @@
   <dimension ref="A1:N63"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="10" customWidth="1" min="1" max="1"/>
-    <col width="10" customWidth="1" min="2" max="2"/>
-    <col width="10" customWidth="1" min="3" max="3"/>
-    <col width="10" customWidth="1" min="4" max="4"/>
-    <col width="10" customWidth="1" min="5" max="5"/>
-    <col width="10" customWidth="1" min="6" max="6"/>
-    <col width="10" customWidth="1" min="7" max="7"/>
-    <col width="10" customWidth="1" min="8" max="8"/>
-    <col width="10" customWidth="1" min="9" max="9"/>
-    <col width="10" customWidth="1" min="10" max="10"/>
-    <col width="10" customWidth="1" min="11" max="11"/>
-    <col width="10" customWidth="1" min="12" max="12"/>
-    <col width="10" customWidth="1" min="13" max="13"/>
-    <col width="10" customWidth="1" min="14" max="14"/>
-    <col width="10" customWidth="1" min="15" max="15"/>
-    <col width="10" customWidth="1" min="16" max="16"/>
-    <col width="10" customWidth="1" min="17" max="17"/>
-    <col width="10" customWidth="1" min="18" max="18"/>
-    <col width="10" customWidth="1" min="19" max="19"/>
+    <col width="9" customWidth="1" min="1" max="1"/>
+    <col width="9" customWidth="1" min="2" max="2"/>
+    <col width="9" customWidth="1" min="3" max="3"/>
+    <col width="9" customWidth="1" min="4" max="4"/>
+    <col width="9" customWidth="1" min="5" max="5"/>
+    <col width="9" customWidth="1" min="6" max="6"/>
+    <col width="9" customWidth="1" min="7" max="7"/>
+    <col width="9" customWidth="1" min="8" max="8"/>
+    <col width="9" customWidth="1" min="9" max="9"/>
+    <col width="9" customWidth="1" min="10" max="10"/>
+    <col width="9" customWidth="1" min="11" max="11"/>
+    <col width="9" customWidth="1" min="12" max="12"/>
+    <col width="9" customWidth="1" min="13" max="13"/>
+    <col width="9" customWidth="1" min="14" max="14"/>
+    <col width="9" customWidth="1" min="15" max="15"/>
+    <col width="9" customWidth="1" min="16" max="16"/>
+    <col width="9" customWidth="1" min="17" max="17"/>
+    <col width="9" customWidth="1" min="18" max="18"/>
+    <col width="9" customWidth="1" min="19" max="19"/>
+    <col width="9" customWidth="1" min="20" max="20"/>
+    <col width="9" customWidth="1" min="21" max="21"/>
   </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1">
@@ -1317,94 +1404,94 @@
       </c>
     </row>
     <row r="55">
-      <c r="A55" t="inlineStr">
+      <c r="F55" t="inlineStr">
         <is>
           <t>Equipo</t>
         </is>
       </c>
-      <c r="B55" t="inlineStr">
+      <c r="G55" t="inlineStr">
         <is>
           <t>OEE %</t>
         </is>
       </c>
     </row>
     <row r="56">
-      <c r="A56" t="inlineStr">
+      <c r="F56" t="inlineStr">
         <is>
           <t>CNC Alpha 01</t>
         </is>
       </c>
-      <c r="B56" t="n">
+      <c r="G56" t="n">
         <v>0.861</v>
       </c>
     </row>
     <row r="57">
-      <c r="A57" t="inlineStr">
+      <c r="F57" t="inlineStr">
         <is>
           <t>CNC Alpha 02</t>
         </is>
       </c>
-      <c r="B57" t="n">
+      <c r="G57" t="n">
         <v>0.842</v>
       </c>
     </row>
     <row r="58">
-      <c r="A58" t="inlineStr">
+      <c r="F58" t="inlineStr">
         <is>
           <t>Torno CNC 03</t>
         </is>
       </c>
-      <c r="B58" t="n">
+      <c r="G58" t="n">
         <v>0.733</v>
       </c>
     </row>
     <row r="59">
-      <c r="A59" t="inlineStr">
+      <c r="F59" t="inlineStr">
         <is>
           <t>Fresadora 04</t>
         </is>
       </c>
-      <c r="B59" t="n">
+      <c r="G59" t="n">
         <v>0.888</v>
       </c>
     </row>
     <row r="60">
-      <c r="A60" t="inlineStr">
+      <c r="F60" t="inlineStr">
         <is>
           <t>Centro Mec. 05</t>
         </is>
       </c>
-      <c r="B60" t="n">
+      <c r="G60" t="n">
         <v>0.828</v>
       </c>
     </row>
     <row r="61">
-      <c r="A61" t="inlineStr">
+      <c r="F61" t="inlineStr">
         <is>
           <t>Torno CNC 06</t>
         </is>
       </c>
-      <c r="B61" t="n">
+      <c r="G61" t="n">
         <v>0.68</v>
       </c>
     </row>
     <row r="62">
-      <c r="A62" t="inlineStr">
+      <c r="F62" t="inlineStr">
         <is>
           <t>Rectificadora 07</t>
         </is>
       </c>
-      <c r="B62" t="n">
+      <c r="G62" t="n">
         <v>0.738</v>
       </c>
     </row>
     <row r="63">
-      <c r="A63" t="inlineStr">
+      <c r="F63" t="inlineStr">
         <is>
           <t>CNC Delta 08</t>
         </is>
       </c>
-      <c r="B63" t="n">
+      <c r="G63" t="n">
         <v>0.914</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Dashboard: reemplaza gráficos openpyxl por imágenes matplotlib con control total de color y layout
</commit_message>
<xml_diff>
--- a/proyectos/excel/gestion-paros-productividad-manufactura/output/Panel_Paros_OEE_Portfolio.xlsx
+++ b/proyectos/excel/gestion-paros-productividad-manufactura/output/Panel_Paros_OEE_Portfolio.xlsx
@@ -435,394 +435,8 @@
 </styleSheet>
 </file>
 
-<file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
-  <chart>
-    <title>
-      <tx>
-        <rich>
-          <a:bodyPr/>
-          <a:p>
-            <a:pPr>
-              <a:defRPr/>
-            </a:pPr>
-            <a:r>
-              <a:t>Pareto de Equipos — Horas de Paro No Programado</a:t>
-            </a:r>
-          </a:p>
-        </rich>
-      </tx>
-    </title>
-    <plotArea>
-      <barChart>
-        <barDir val="col"/>
-        <grouping val="clustered"/>
-        <ser>
-          <idx val="0"/>
-          <order val="0"/>
-          <tx>
-            <strRef>
-              <f>'Dashboard'!B42</f>
-            </strRef>
-          </tx>
-          <spPr>
-            <a:solidFill>
-              <a:srgbClr val="2E75B6"/>
-            </a:solidFill>
-            <a:ln>
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <cat>
-            <numRef>
-              <f>'Dashboard'!$A$43:$A$50</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'Dashboard'!$B$43:$B$50</f>
-            </numRef>
-          </val>
-        </ser>
-        <gapWidth val="150"/>
-        <axId val="10"/>
-        <axId val="100"/>
-      </barChart>
-      <lineChart>
-        <grouping val="standard"/>
-        <ser>
-          <idx val="1"/>
-          <order val="1"/>
-          <tx>
-            <strRef>
-              <f>'Dashboard'!C42</f>
-            </strRef>
-          </tx>
-          <spPr>
-            <a:ln w="20000">
-              <a:solidFill>
-                <a:srgbClr val="ED7D31"/>
-              </a:solidFill>
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <marker>
-            <symbol val="none"/>
-            <spPr>
-              <a:ln>
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </spPr>
-          </marker>
-          <cat>
-            <numRef>
-              <f>'Dashboard'!$A$43:$A$50</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'Dashboard'!$C$43:$C$50</f>
-            </numRef>
-          </val>
-        </ser>
-        <axId val="10"/>
-        <axId val="200"/>
-      </lineChart>
-      <catAx>
-        <axId val="10"/>
-        <scaling>
-          <orientation val="minMax"/>
-        </scaling>
-        <axPos val="l"/>
-        <title>
-          <tx>
-            <rich>
-              <a:bodyPr/>
-              <a:p>
-                <a:pPr>
-                  <a:defRPr/>
-                </a:pPr>
-                <a:r>
-                  <a:t>Equipo</a:t>
-                </a:r>
-              </a:p>
-            </rich>
-          </tx>
-        </title>
-        <majorTickMark val="none"/>
-        <minorTickMark val="none"/>
-        <crossAx val="100"/>
-        <lblOffset val="100"/>
-      </catAx>
-      <valAx>
-        <axId val="100"/>
-        <scaling>
-          <orientation val="minMax"/>
-        </scaling>
-        <axPos val="l"/>
-        <majorGridlines/>
-        <title>
-          <tx>
-            <rich>
-              <a:bodyPr/>
-              <a:p>
-                <a:pPr>
-                  <a:defRPr/>
-                </a:pPr>
-                <a:r>
-                  <a:t>Horas</a:t>
-                </a:r>
-              </a:p>
-            </rich>
-          </tx>
-        </title>
-        <majorTickMark val="none"/>
-        <minorTickMark val="none"/>
-        <crossAx val="10"/>
-      </valAx>
-      <valAx>
-        <axId val="200"/>
-        <scaling>
-          <orientation val="minMax"/>
-        </scaling>
-        <axPos val="l"/>
-        <majorGridlines/>
-        <title>
-          <tx>
-            <rich>
-              <a:bodyPr/>
-              <a:p>
-                <a:pPr>
-                  <a:defRPr/>
-                </a:pPr>
-                <a:r>
-                  <a:t>% Acumulado</a:t>
-                </a:r>
-              </a:p>
-            </rich>
-          </tx>
-        </title>
-        <numFmt formatCode="0%" sourceLinked="0"/>
-        <majorTickMark val="none"/>
-        <minorTickMark val="none"/>
-        <crossAx val="10"/>
-        <crosses val="max"/>
-      </valAx>
-    </plotArea>
-    <legend>
-      <legendPos val="r"/>
-    </legend>
-    <plotVisOnly val="1"/>
-    <dispBlanksAs val="gap"/>
-  </chart>
-</chartSpace>
-</file>
-
-<file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
-  <chart>
-    <title>
-      <tx>
-        <rich>
-          <a:bodyPr/>
-          <a:p>
-            <a:pPr>
-              <a:defRPr/>
-            </a:pPr>
-            <a:r>
-              <a:t>OEE por Equipo — Eficiencia General 2024</a:t>
-            </a:r>
-          </a:p>
-        </rich>
-      </tx>
-    </title>
-    <plotArea>
-      <barChart>
-        <barDir val="bar"/>
-        <grouping val="clustered"/>
-        <ser>
-          <idx val="0"/>
-          <order val="0"/>
-          <tx>
-            <strRef>
-              <f>'Dashboard'!G55</f>
-            </strRef>
-          </tx>
-          <spPr>
-            <a:ln>
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <dPt>
-            <idx val="0"/>
-            <spPr>
-              <a:solidFill>
-                <a:srgbClr val="70AD47"/>
-              </a:solidFill>
-              <a:ln>
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </spPr>
-          </dPt>
-          <dPt>
-            <idx val="1"/>
-            <spPr>
-              <a:solidFill>
-                <a:srgbClr val="FFD966"/>
-              </a:solidFill>
-              <a:ln>
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </spPr>
-          </dPt>
-          <dPt>
-            <idx val="2"/>
-            <spPr>
-              <a:solidFill>
-                <a:srgbClr val="FFD966"/>
-              </a:solidFill>
-              <a:ln>
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </spPr>
-          </dPt>
-          <dPt>
-            <idx val="3"/>
-            <spPr>
-              <a:solidFill>
-                <a:srgbClr val="70AD47"/>
-              </a:solidFill>
-              <a:ln>
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </spPr>
-          </dPt>
-          <dPt>
-            <idx val="4"/>
-            <spPr>
-              <a:solidFill>
-                <a:srgbClr val="FFD966"/>
-              </a:solidFill>
-              <a:ln>
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </spPr>
-          </dPt>
-          <dPt>
-            <idx val="5"/>
-            <spPr>
-              <a:solidFill>
-                <a:srgbClr val="FFD966"/>
-              </a:solidFill>
-              <a:ln>
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </spPr>
-          </dPt>
-          <dPt>
-            <idx val="6"/>
-            <spPr>
-              <a:solidFill>
-                <a:srgbClr val="FFD966"/>
-              </a:solidFill>
-              <a:ln>
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </spPr>
-          </dPt>
-          <dPt>
-            <idx val="7"/>
-            <spPr>
-              <a:solidFill>
-                <a:srgbClr val="70AD47"/>
-              </a:solidFill>
-              <a:ln>
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </spPr>
-          </dPt>
-          <cat>
-            <numRef>
-              <f>'Dashboard'!$F$56:$F$63</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'Dashboard'!$G$56:$G$63</f>
-            </numRef>
-          </val>
-        </ser>
-        <gapWidth val="150"/>
-        <axId val="10"/>
-        <axId val="100"/>
-      </barChart>
-      <catAx>
-        <axId val="10"/>
-        <scaling>
-          <orientation val="minMax"/>
-          <max val="1"/>
-          <min val="0.6"/>
-        </scaling>
-        <axPos val="l"/>
-        <title>
-          <tx>
-            <rich>
-              <a:bodyPr/>
-              <a:p>
-                <a:pPr>
-                  <a:defRPr/>
-                </a:pPr>
-                <a:r>
-                  <a:t>OEE %</a:t>
-                </a:r>
-              </a:p>
-            </rich>
-          </tx>
-        </title>
-        <numFmt formatCode="0%" sourceLinked="0"/>
-        <majorTickMark val="none"/>
-        <minorTickMark val="none"/>
-        <crossAx val="100"/>
-        <lblOffset val="100"/>
-      </catAx>
-      <valAx>
-        <axId val="100"/>
-        <scaling>
-          <orientation val="minMax"/>
-        </scaling>
-        <axPos val="l"/>
-        <majorGridlines/>
-        <title>
-          <tx>
-            <rich>
-              <a:bodyPr/>
-              <a:p>
-                <a:pPr>
-                  <a:defRPr/>
-                </a:pPr>
-                <a:r>
-                  <a:t>Equipo</a:t>
-                </a:r>
-              </a:p>
-            </rich>
-          </tx>
-        </title>
-        <majorTickMark val="none"/>
-        <minorTickMark val="none"/>
-        <crossAx val="10"/>
-      </valAx>
-    </plotArea>
-    <legend>
-      <legendPos val="r"/>
-    </legend>
-    <plotVisOnly val="1"/>
-    <dispBlanksAs val="gap"/>
-  </chart>
-</chartSpace>
-</file>
-
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
       <col>1</col>
@@ -830,19 +444,22 @@
       <row>6</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="7200000" cy="5040000"/>
-    <graphicFrame>
-      <nvGraphicFramePr>
-        <cNvPr id="1" name="Chart 1"/>
-        <cNvGraphicFramePr/>
-      </nvGraphicFramePr>
-      <xfrm/>
-      <a:graphic>
-        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart r:id="rId1"/>
-        </a:graphicData>
-      </a:graphic>
-    </graphicFrame>
+    <ext cx="5048250" cy="3429000"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="1" name="Image 1" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
     <clientData/>
   </oneCellAnchor>
   <oneCellAnchor>
@@ -852,19 +469,22 @@
       <row>6</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="7920000" cy="5040000"/>
-    <graphicFrame>
-      <nvGraphicFramePr>
-        <cNvPr id="2" name="Chart 2"/>
-        <cNvGraphicFramePr/>
-      </nvGraphicFramePr>
-      <xfrm/>
-      <a:graphic>
-        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart r:id="rId2"/>
-        </a:graphicData>
-      </a:graphic>
-    </graphicFrame>
+    <ext cx="5048250" cy="3429000"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="2" name="Image 2" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId2"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
     <clientData/>
   </oneCellAnchor>
 </wsDr>
@@ -1179,7 +799,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N63"/>
+  <dimension ref="A1:N31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -1280,219 +900,6 @@
         <is>
           <t>Datos sintéticos con distribuciones realistas del sector manufacturero — Portfolio de Datos y Analítica | Luciano Villagrán</t>
         </is>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" t="inlineStr">
-        <is>
-          <t>Equipo</t>
-        </is>
-      </c>
-      <c r="B42" t="inlineStr">
-        <is>
-          <t>Horas NP</t>
-        </is>
-      </c>
-      <c r="C42" t="inlineStr">
-        <is>
-          <t>% Acum.</t>
-        </is>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" t="inlineStr">
-        <is>
-          <t>Torno CNC 06</t>
-        </is>
-      </c>
-      <c r="B43" t="n">
-        <v>273.9</v>
-      </c>
-      <c r="C43" t="n">
-        <v>0.254</v>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" t="inlineStr">
-        <is>
-          <t>Rectificadora 07</t>
-        </is>
-      </c>
-      <c r="B44" t="n">
-        <v>213.7</v>
-      </c>
-      <c r="C44" t="n">
-        <v>0.452</v>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" t="inlineStr">
-        <is>
-          <t>Torno CNC 03</t>
-        </is>
-      </c>
-      <c r="B45" t="n">
-        <v>202.8</v>
-      </c>
-      <c r="C45" t="n">
-        <v>0.64</v>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" t="inlineStr">
-        <is>
-          <t>Fresadora 04</t>
-        </is>
-      </c>
-      <c r="B46" t="n">
-        <v>104.1</v>
-      </c>
-      <c r="C46" t="n">
-        <v>0.736</v>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" t="inlineStr">
-        <is>
-          <t>CNC Alpha 01</t>
-        </is>
-      </c>
-      <c r="B47" t="n">
-        <v>101.6</v>
-      </c>
-      <c r="C47" t="n">
-        <v>0.83</v>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" t="inlineStr">
-        <is>
-          <t>Centro Mec. 05</t>
-        </is>
-      </c>
-      <c r="B48" t="n">
-        <v>87.59999999999999</v>
-      </c>
-      <c r="C48" t="n">
-        <v>0.912</v>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" t="inlineStr">
-        <is>
-          <t>CNC Alpha 02</t>
-        </is>
-      </c>
-      <c r="B49" t="n">
-        <v>73</v>
-      </c>
-      <c r="C49" t="n">
-        <v>0.979</v>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50" t="inlineStr">
-        <is>
-          <t>CNC Delta 08</t>
-        </is>
-      </c>
-      <c r="B50" t="n">
-        <v>22.4</v>
-      </c>
-      <c r="C50" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="55">
-      <c r="F55" t="inlineStr">
-        <is>
-          <t>Equipo</t>
-        </is>
-      </c>
-      <c r="G55" t="inlineStr">
-        <is>
-          <t>OEE %</t>
-        </is>
-      </c>
-    </row>
-    <row r="56">
-      <c r="F56" t="inlineStr">
-        <is>
-          <t>CNC Alpha 01</t>
-        </is>
-      </c>
-      <c r="G56" t="n">
-        <v>0.861</v>
-      </c>
-    </row>
-    <row r="57">
-      <c r="F57" t="inlineStr">
-        <is>
-          <t>CNC Alpha 02</t>
-        </is>
-      </c>
-      <c r="G57" t="n">
-        <v>0.842</v>
-      </c>
-    </row>
-    <row r="58">
-      <c r="F58" t="inlineStr">
-        <is>
-          <t>Torno CNC 03</t>
-        </is>
-      </c>
-      <c r="G58" t="n">
-        <v>0.733</v>
-      </c>
-    </row>
-    <row r="59">
-      <c r="F59" t="inlineStr">
-        <is>
-          <t>Fresadora 04</t>
-        </is>
-      </c>
-      <c r="G59" t="n">
-        <v>0.888</v>
-      </c>
-    </row>
-    <row r="60">
-      <c r="F60" t="inlineStr">
-        <is>
-          <t>Centro Mec. 05</t>
-        </is>
-      </c>
-      <c r="G60" t="n">
-        <v>0.828</v>
-      </c>
-    </row>
-    <row r="61">
-      <c r="F61" t="inlineStr">
-        <is>
-          <t>Torno CNC 06</t>
-        </is>
-      </c>
-      <c r="G61" t="n">
-        <v>0.68</v>
-      </c>
-    </row>
-    <row r="62">
-      <c r="F62" t="inlineStr">
-        <is>
-          <t>Rectificadora 07</t>
-        </is>
-      </c>
-      <c r="G62" t="n">
-        <v>0.738</v>
-      </c>
-    </row>
-    <row r="63">
-      <c r="F63" t="inlineStr">
-        <is>
-          <t>CNC Delta 08</t>
-        </is>
-      </c>
-      <c r="G63" t="n">
-        <v>0.914</v>
       </c>
     </row>
   </sheetData>

</xml_diff>